<commit_message>
Updated spreadsheet: STM32H743X pinout
</commit_message>
<xml_diff>
--- a/design/PINOUT_STM32.xlsx
+++ b/design/PINOUT_STM32.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{2D69C361-96F9-440C-81E4-FCEE4764BAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C69AED7E-D364-4905-A5EA-459E7F0B23B2}"/>
+  <xr:revisionPtr revIDLastSave="186" documentId="8_{2D69C361-96F9-440C-81E4-FCEE4764BAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1166490E-239C-4C50-BA09-17ABD3CACE00}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{CD38DF22-F41A-4FF5-9B41-74C32AB1E5AF}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="150">
   <si>
     <t>Driver 1</t>
   </si>
@@ -487,6 +487,93 @@
   </si>
   <si>
     <t>PB9</t>
+  </si>
+  <si>
+    <t>Rotary Encoder</t>
+  </si>
+  <si>
+    <t>DT</t>
+  </si>
+  <si>
+    <t>CLK</t>
+  </si>
+  <si>
+    <t>SW</t>
+  </si>
+  <si>
+    <t>PD3</t>
+  </si>
+  <si>
+    <t>PD4</t>
+  </si>
+  <si>
+    <t>PI1</t>
+  </si>
+  <si>
+    <t>pull-up</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>Heartbeat LED</t>
+  </si>
+  <si>
+    <t>TIM1_CH1</t>
+  </si>
+  <si>
+    <t>TIM1_CH4</t>
+  </si>
+  <si>
+    <t>TIM2_CH4</t>
+  </si>
+  <si>
+    <t>TIM2_CH2</t>
+  </si>
+  <si>
+    <t>TIM2_CH3</t>
+  </si>
+  <si>
+    <t>TIM3_CH1</t>
+  </si>
+  <si>
+    <t>NEOPIXEL_D</t>
+  </si>
+  <si>
+    <t>COM</t>
+  </si>
+  <si>
+    <t>I2C1_SCL</t>
+  </si>
+  <si>
+    <t>I2C1_SDA</t>
+  </si>
+  <si>
+    <t>PA9</t>
+  </si>
+  <si>
+    <t>PA10</t>
+  </si>
+  <si>
+    <t>TX</t>
+  </si>
+  <si>
+    <t>RX</t>
+  </si>
+  <si>
+    <t>USART1_TX</t>
+  </si>
+  <si>
+    <t>USART1_RX</t>
+  </si>
+  <si>
+    <t>PC6</t>
+  </si>
+  <si>
+    <t>PD12</t>
+  </si>
+  <si>
+    <t>TIM4_CH1</t>
   </si>
 </sst>
 </file>
@@ -1260,10 +1347,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79292074-276B-4B71-8582-2138DE8711E5}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" style="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10" style="13" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" style="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.28515625" style="13" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -1394,7 +1481,9 @@
       <c r="A9" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>131</v>
+      </c>
       <c r="C9" s="3" t="s">
         <v>67</v>
       </c>
@@ -1448,7 +1537,9 @@
       <c r="A15" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="10"/>
+      <c r="B15" s="10" t="s">
+        <v>132</v>
+      </c>
       <c r="C15" s="3" t="s">
         <v>73</v>
       </c>
@@ -1457,7 +1548,9 @@
       <c r="A16" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="10" t="s">
+        <v>133</v>
+      </c>
       <c r="C16" s="3" t="s">
         <v>74</v>
       </c>
@@ -1513,7 +1606,9 @@
       <c r="A22" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="10"/>
+      <c r="B22" s="10" t="s">
+        <v>134</v>
+      </c>
       <c r="C22" s="3" t="s">
         <v>80</v>
       </c>
@@ -1522,7 +1617,9 @@
       <c r="A23" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="10"/>
+      <c r="B23" s="10" t="s">
+        <v>135</v>
+      </c>
       <c r="C23" s="3" t="s">
         <v>81</v>
       </c>
@@ -1565,7 +1662,9 @@
       <c r="A28" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B28" s="10"/>
+      <c r="B28" s="10" t="s">
+        <v>140</v>
+      </c>
       <c r="C28" s="10" t="s">
         <v>35</v>
       </c>
@@ -1574,45 +1673,138 @@
       <c r="A29" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B29" s="10"/>
+      <c r="B29" s="10" t="s">
+        <v>139</v>
+      </c>
       <c r="C29" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
+      <c r="A30" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" s="18"/>
+      <c r="C30" s="19"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
+      <c r="A31" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
+      <c r="A32" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
+      <c r="A33" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
+      <c r="A34" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="B34" s="18"/>
+      <c r="C34" s="19"/>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
+      <c r="A35" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B38" s="18"/>
+      <c r="C38" s="19"/>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="10"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A38:C38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Pinout mapping for STM32H743XIH6
</commit_message>
<xml_diff>
--- a/design/PINOUT_STM32.xlsx
+++ b/design/PINOUT_STM32.xlsx
@@ -1004,8 +1004,8 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1759,6 +1759,7 @@
     <mergeCell ref="A38:C38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update Agriculture edges: Pollution
</commit_message>
<xml_diff>
--- a/design/PINOUT_STM32.xlsx
+++ b/design/PINOUT_STM32.xlsx
@@ -8,18 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="190" documentId="8_{2D69C361-96F9-440C-81E4-FCEE4764BAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{793F110C-9BF5-4633-AD65-2709CC83392C}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="8_{2D69C361-96F9-440C-81E4-FCEE4764BAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B786F869-0D28-410F-B349-F9E3938E24CE}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{CD38DF22-F41A-4FF5-9B41-74C32AB1E5AF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CD38DF22-F41A-4FF5-9B41-74C32AB1E5AF}"/>
   </bookViews>
   <sheets>
     <sheet name="STM32H743XIH6" sheetId="1" r:id="rId1"/>
     <sheet name="TB6612FNG" sheetId="2" r:id="rId2"/>
     <sheet name="PCA9548a" sheetId="3" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
@@ -45,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="163">
   <si>
     <t>Driver 1</t>
   </si>
@@ -68,27 +65,15 @@
     <t>A01</t>
   </si>
   <si>
-    <t>Slider 5 +</t>
-  </si>
-  <si>
     <t>A02</t>
   </si>
   <si>
-    <t>Slider 5 -</t>
-  </si>
-  <si>
     <t>B02</t>
   </si>
   <si>
-    <t>Slider 4 -</t>
-  </si>
-  <si>
     <t>B01</t>
   </si>
   <si>
-    <t>Slider 4 +</t>
-  </si>
-  <si>
     <t>PWMA</t>
   </si>
   <si>
@@ -116,18 +101,6 @@
     <t>3V3</t>
   </si>
   <si>
-    <t>Slider 3 +</t>
-  </si>
-  <si>
-    <t>Slider 3 -</t>
-  </si>
-  <si>
-    <t>Slider 2 -</t>
-  </si>
-  <si>
-    <t>Slider 2 +</t>
-  </si>
-  <si>
     <t>Driver 3</t>
   </si>
   <si>
@@ -137,9 +110,6 @@
     <t>Slider 1+</t>
   </si>
   <si>
-    <t>Slider 1 -</t>
-  </si>
-  <si>
     <t>VIN</t>
   </si>
   <si>
@@ -164,9 +134,6 @@
     <t>SD6</t>
   </si>
   <si>
-    <t>3v3</t>
-  </si>
-  <si>
     <t>RST</t>
   </si>
   <si>
@@ -185,43 +152,28 @@
     <t>SC4</t>
   </si>
   <si>
-    <t>OLED5</t>
-  </si>
-  <si>
     <t>A2</t>
   </si>
   <si>
     <t>SD4</t>
   </si>
   <si>
-    <t>OLED1</t>
-  </si>
-  <si>
     <t>SD0</t>
   </si>
   <si>
     <t>SC3</t>
   </si>
   <si>
-    <t>OLED4</t>
-  </si>
-  <si>
     <t>SC0</t>
   </si>
   <si>
     <t>SD3</t>
   </si>
   <si>
-    <t>OLED2</t>
-  </si>
-  <si>
     <t>SD1</t>
   </si>
   <si>
     <t>SC2</t>
-  </si>
-  <si>
-    <t>OLED3</t>
   </si>
   <si>
     <t>SC1</t>
@@ -575,6 +527,90 @@
   </si>
   <si>
     <t>TIM4_CH1</t>
+  </si>
+  <si>
+    <t>RESET</t>
+  </si>
+  <si>
+    <t>PB8</t>
+  </si>
+  <si>
+    <t>RESET_PCA9548A</t>
+  </si>
+  <si>
+    <t>OLED1_SDA</t>
+  </si>
+  <si>
+    <t>OLED1_SCL</t>
+  </si>
+  <si>
+    <t>OLED2_SDA</t>
+  </si>
+  <si>
+    <t>OLED2_SCL</t>
+  </si>
+  <si>
+    <t>OLED5_SCL</t>
+  </si>
+  <si>
+    <t>OLED5_SDA</t>
+  </si>
+  <si>
+    <t>OLED4_SCL</t>
+  </si>
+  <si>
+    <t>OLED4_SDA</t>
+  </si>
+  <si>
+    <t>OLED3_SCL</t>
+  </si>
+  <si>
+    <t>OLED3_SDA</t>
+  </si>
+  <si>
+    <t>SWDIO</t>
+  </si>
+  <si>
+    <t>SWCLK</t>
+  </si>
+  <si>
+    <t>PA13</t>
+  </si>
+  <si>
+    <t>PA14</t>
+  </si>
+  <si>
+    <t>SWDIO_DEBUG</t>
+  </si>
+  <si>
+    <t>SWCLK_DEBUG</t>
+  </si>
+  <si>
+    <t>Slider 5+</t>
+  </si>
+  <si>
+    <t>Slider 5-</t>
+  </si>
+  <si>
+    <t>Slider 1-</t>
+  </si>
+  <si>
+    <t>Slider 2-</t>
+  </si>
+  <si>
+    <t>Slider 2+</t>
+  </si>
+  <si>
+    <t>Slider 3+</t>
+  </si>
+  <si>
+    <t>Slider 3-</t>
+  </si>
+  <si>
+    <t>Slider 4-</t>
+  </si>
+  <si>
+    <t>Slider 4+</t>
   </si>
 </sst>
 </file>
@@ -935,8 +971,8 @@
       <xdr:rowOff>81430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>8493</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>208518</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>10646</xdr:rowOff>
     </xdr:to>
@@ -978,37 +1014,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="esp32 (v2)"/>
-      <sheetName val="TB6612FNG"/>
-      <sheetName val="pca9548a"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>GND</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>GND</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1332,11 +1337,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79292074-276B-4B71-8582-2138DE8711E5}">
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" style="10" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.85546875" customWidth="1"/>
@@ -1345,418 +1350,441 @@
   <sheetData>
     <row r="1" spans="1:11" s="8" customFormat="1">
       <c r="A1" s="11" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="H1" s="12"/>
       <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="7" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="7" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="7" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="7" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="13" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="15"/>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="9" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="2" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="2" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="2" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="2" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="2" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="2" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="2" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="2" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="2" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="2" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="2" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="2" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="2" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="2" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="2" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="2" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="13" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="15"/>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="7" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="7" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="15"/>
+      <c r="A30" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>122</v>
-      </c>
+      <c r="A31" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B31" s="14"/>
+      <c r="C31" s="15"/>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="7" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="7" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:3">
-      <c r="A34" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="15"/>
+      <c r="A34" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="35" spans="1:3">
-      <c r="A35" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>130</v>
-      </c>
+      <c r="A35" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="14"/>
+      <c r="C35" s="15"/>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="7" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>137</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:3">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
+      <c r="A37" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="38" spans="1:3">
-      <c r="A38" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B38" s="14"/>
-      <c r="C38" s="15"/>
+      <c r="A38" s="7"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>143</v>
-      </c>
+      <c r="A39" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="B39" s="14"/>
+      <c r="C39" s="15"/>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="7" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
+      <c r="A41" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="7"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
+      <c r="A42" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
+      <c r="A43" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="7"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A39:C39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -1805,9 +1833,8 @@
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="str">
-        <f>'[1]esp32 (v2)'!A12</f>
-        <v>GND</v>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="9" customHeight="1">
@@ -1815,83 +1842,103 @@
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="9" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>9</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="9" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>11</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="9" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>13</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="9" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="str">
-        <f>'[1]esp32 (v2)'!A13</f>
-        <v>GND</v>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="9" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <f>STM32H743XIH6!A9</f>
+        <v>PA8</v>
+      </c>
     </row>
     <row r="11" spans="1:2" ht="9" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <f>STM32H743XIH6!A10</f>
+        <v>PC5</v>
+      </c>
     </row>
     <row r="12" spans="1:2" ht="9" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <f>STM32H743XIH6!A11</f>
+        <v>PB0</v>
+      </c>
     </row>
     <row r="13" spans="1:2" ht="9" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="B13" s="2" t="str">
+        <f>STM32H743XIH6!A12</f>
+        <v>PE5</v>
+      </c>
     </row>
     <row r="14" spans="1:2" ht="9" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="B14" s="2" t="str">
+        <f>STM32H743XIH6!A13</f>
+        <v>PA5</v>
+      </c>
     </row>
     <row r="15" spans="1:2" ht="9" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <f>STM32H743XIH6!A14</f>
+        <v>PA4</v>
+      </c>
     </row>
     <row r="16" spans="1:2" ht="9" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="2"/>
+        <v>16</v>
+      </c>
+      <c r="B16" s="2" t="str">
+        <f>STM32H743XIH6!A15</f>
+        <v>PA11</v>
+      </c>
     </row>
     <row r="17" spans="1:2" ht="9" customHeight="1">
       <c r="A17" s="2" t="s">
@@ -1903,7 +1950,7 @@
     </row>
     <row r="18" spans="1:2" ht="9" customHeight="1">
       <c r="A18" s="16" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B18" s="16"/>
     </row>
@@ -1921,16 +1968,15 @@
         <v>3</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="9" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="2" t="str">
-        <f>'[1]esp32 (v2)'!A13</f>
-        <v>GND</v>
+      <c r="B21" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="9" customHeight="1">
@@ -1938,96 +1984,115 @@
         <v>6</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>23</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="9" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>24</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="9" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>25</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="9" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>26</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="9" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B26" s="2" t="str">
-        <f>'[1]esp32 (v2)'!A13</f>
-        <v>GND</v>
+      <c r="B26" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="9" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B27" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <f>STM32H743XIH6!A16</f>
+        <v>PB11</v>
+      </c>
     </row>
     <row r="28" spans="1:2" ht="9" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <f>STM32H743XIH6!A17</f>
+        <v>PA7</v>
+      </c>
     </row>
     <row r="29" spans="1:2" ht="9" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B29" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <f>STM32H743XIH6!A18</f>
+        <v>PB2</v>
+      </c>
     </row>
     <row r="30" spans="1:2" ht="9" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B30" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="B30" s="2" t="str">
+        <f>STM32H743XIH6!A19</f>
+        <v>PE5</v>
+      </c>
     </row>
     <row r="31" spans="1:2" ht="9" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="B31" s="2" t="str">
+        <f>STM32H743XIH6!A20</f>
+        <v>PE3</v>
+      </c>
     </row>
     <row r="32" spans="1:2" ht="9" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="B32" s="2" t="str">
+        <f>STM32H743XIH6!A21</f>
+        <v>PB9</v>
+      </c>
     </row>
     <row r="33" spans="1:2" ht="9" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="2"/>
+        <v>16</v>
+      </c>
+      <c r="B33" s="2" t="str">
+        <f>STM32H743XIH6!A22</f>
+        <v>PA1</v>
+      </c>
     </row>
     <row r="34" spans="1:2" ht="9" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="2" t="str">
-        <f>'[1]esp32 (v2)'!A13</f>
-        <v>GND</v>
+      <c r="B34" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="9" customHeight="1">
       <c r="A35" s="16" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B35" s="16"/>
     </row>
@@ -2045,7 +2110,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="9" customHeight="1">
@@ -2061,31 +2126,31 @@
         <v>6</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>29</v>
+        <v>154</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="9" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>30</v>
+        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="9" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="9" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="9" customHeight="1">
@@ -2098,59 +2163,70 @@
     </row>
     <row r="44" spans="1:2" ht="9" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B44" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="B44" s="2" t="str">
+        <f>STM32H743XIH6!A23</f>
+        <v>PA2</v>
+      </c>
     </row>
     <row r="45" spans="1:2" ht="9" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B45" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B45" s="2" t="str">
+        <f>STM32H743XIH6!A24</f>
+        <v>PE4</v>
+      </c>
     </row>
     <row r="46" spans="1:2" ht="9" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="B46" s="2" t="str">
+        <f>STM32H743XIH6!A25</f>
+        <v>PC1</v>
+      </c>
     </row>
     <row r="47" spans="1:2" ht="9" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B47" s="2"/>
+        <v>13</v>
+      </c>
+      <c r="B47" s="2" t="str">
+        <f>STM32H743XIH6!A26</f>
+        <v>PE5</v>
+      </c>
     </row>
     <row r="48" spans="1:2" ht="9" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="9" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="9" customHeight="1">
       <c r="A50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="9" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B51" s="2">
-        <f>'[1]esp32 (v2)'!A43</f>
-        <v>0</v>
+      <c r="B51" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2174,8 +2250,8 @@
   <dimension ref="A2:E31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="15.75" thickBot="1"/>
@@ -2184,14 +2260,14 @@
         <v>4</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2203,51 +2279,58 @@
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="3"/>
+      <c r="A5" s="3" t="str">
+        <f>STM32H743XIH6!A28</f>
+        <v>PB7</v>
+      </c>
       <c r="B5" s="5" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="3"/>
+      <c r="A6" s="3" t="str">
+        <f>STM32H743XIH6!A29</f>
+        <v>PB6</v>
+      </c>
       <c r="B6" s="5" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="3" t="s">
-        <v>39</v>
+      <c r="A7" s="3" t="str">
+        <f>STM32H743XIH6!A30</f>
+        <v>PB8</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2255,14 +2338,14 @@
         <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2270,14 +2353,14 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>46</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2285,79 +2368,79 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>46</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="3" t="s">
-        <v>49</v>
+        <v>138</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>52</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
-        <v>49</v>
+        <v>139</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>52</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="3" t="s">
-        <v>55</v>
+        <v>140</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>58</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1">
       <c r="A14" s="3" t="s">
-        <v>55</v>
+        <v>141</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>58</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="44.1" customHeight="1">
       <c r="B31" s="17" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>

</xml_diff>